<commit_message>
Header is 'Total Score (0–3)'; rooms are individual scoring columns (drop per-room SUM)
</commit_message>
<xml_diff>
--- a/template/6S-Audit-Template.xlsx
+++ b/template/6S-Audit-Template.xlsx
@@ -1050,7 +1050,7 @@
       </c>
       <c r="D7" s="17" t="inlineStr">
         <is>
-          <t>Score
+          <t>Total Score
 (0–3)</t>
         </is>
       </c>
@@ -1936,7 +1936,7 @@
       </c>
       <c r="D7" s="17" t="inlineStr">
         <is>
-          <t>Score
+          <t>Total Score
 (0–3)</t>
         </is>
       </c>

</xml_diff>